<commit_message>
test with pro-forma data
</commit_message>
<xml_diff>
--- a/active_portfolio.xlsx
+++ b/active_portfolio.xlsx
@@ -1,34 +1,106 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daivieth/Documents/_G8I/Development/IVP-Portfolio-Management-Utils/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74156DAC-B813-8940-BFCE-25B773B88714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+  <si>
+    <t>ticker</t>
+  </si>
+  <si>
+    <t>quantity</t>
+  </si>
+  <si>
+    <t>QAN.AX</t>
+  </si>
+  <si>
+    <t>HUB.AX</t>
+  </si>
+  <si>
+    <t>ORG.AX</t>
+  </si>
+  <si>
+    <t>GNP.AX</t>
+  </si>
+  <si>
+    <t>MTS.AX</t>
+  </si>
+  <si>
+    <t>QBE.AX</t>
+  </si>
+  <si>
+    <t>IAG.AX</t>
+  </si>
+  <si>
+    <t>PRN.AX</t>
+  </si>
+  <si>
+    <t>ABB.AX</t>
+  </si>
+  <si>
+    <t>SGLLV.AX</t>
+  </si>
+  <si>
+    <t>UNI.AX</t>
+  </si>
+  <si>
+    <t>ORI.AX</t>
+  </si>
+  <si>
+    <t>CAR.AX</t>
+  </si>
+  <si>
+    <t>TCO.AX</t>
+  </si>
+  <si>
+    <t>PPS.AX</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,81 +118,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -408,65 +423,385 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B78"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>ticker</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>quantity</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>AAPL</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="1">
+        <v>972</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B4" s="1">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1">
+        <v>3289</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="1">
+        <v>2300</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="1">
+        <v>1823</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="1">
+        <v>2663</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1">
+        <v>3474</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="1">
+        <v>1088</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="1">
+        <v>9949</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" s="1">
+        <v>8634</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>MSFT</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>NVDA</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>TSLA</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>15</v>
-      </c>
+      <c r="B13" s="1">
+        <v>4750</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B14" s="1">
+        <v>2003</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15" s="1">
+        <v>7348</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="1">
+        <v>33578</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" s="1"/>
+      <c r="B26" s="1"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="1"/>
+      <c r="B27" s="1"/>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1"/>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1"/>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" s="1"/>
+      <c r="B34" s="1"/>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" s="1"/>
+      <c r="B35" s="1"/>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" s="1"/>
+      <c r="B36" s="1"/>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37" s="1"/>
+      <c r="B37" s="1"/>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" s="1"/>
+      <c r="B38" s="1"/>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" s="1"/>
+      <c r="B39" s="1"/>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" s="1"/>
+      <c r="B40" s="1"/>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" s="1"/>
+      <c r="B41" s="1"/>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" s="1"/>
+      <c r="B42" s="1"/>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" s="1"/>
+      <c r="B43" s="1"/>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44" s="1"/>
+      <c r="B44" s="1"/>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" s="1"/>
+      <c r="B45" s="1"/>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" s="1"/>
+      <c r="B46" s="1"/>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" s="1"/>
+      <c r="B47" s="1"/>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48" s="1"/>
+      <c r="B48" s="1"/>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" s="1"/>
+      <c r="B49" s="1"/>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" s="1"/>
+      <c r="B50" s="1"/>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51" s="1"/>
+      <c r="B51" s="1"/>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A52" s="1"/>
+      <c r="B52" s="1"/>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53" s="1"/>
+      <c r="B53" s="1"/>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54" s="1"/>
+      <c r="B54" s="1"/>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" s="1"/>
+      <c r="B55" s="1"/>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56" s="1"/>
+      <c r="B56" s="1"/>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57" s="1"/>
+      <c r="B57" s="1"/>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" s="1"/>
+      <c r="B58" s="1"/>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" s="1"/>
+      <c r="B59" s="1"/>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60" s="1"/>
+      <c r="B60" s="1"/>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" s="1"/>
+      <c r="B61" s="1"/>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62" s="1"/>
+      <c r="B62" s="1"/>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A63" s="1"/>
+      <c r="B63" s="1"/>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A64" s="1"/>
+      <c r="B64" s="1"/>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A65" s="1"/>
+      <c r="B65" s="1"/>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A66" s="1"/>
+      <c r="B66" s="1"/>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A67" s="1"/>
+      <c r="B67" s="1"/>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A68" s="1"/>
+      <c r="B68" s="1"/>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A69" s="1"/>
+      <c r="B69" s="1"/>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A70" s="1"/>
+      <c r="B70" s="1"/>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A71" s="1"/>
+      <c r="B71" s="1"/>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A72" s="1"/>
+      <c r="B72" s="1"/>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A73" s="1"/>
+      <c r="B73" s="1"/>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74" s="1"/>
+      <c r="B74" s="1"/>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A75" s="1"/>
+      <c r="B75" s="1"/>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A76" s="1"/>
+      <c r="B76" s="1"/>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A77" s="1"/>
+      <c r="B77" s="1"/>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A78" s="1"/>
+      <c r="B78" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
adding the sector/industry exposure analysis
</commit_message>
<xml_diff>
--- a/active_portfolio.xlsx
+++ b/active_portfolio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daivieth/Documents/_G8I/Development/IVP-Portfolio-Management-Utils/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74156DAC-B813-8940-BFCE-25B773B88714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B25A1895-5226-B544-B641-3B1BE21E8E2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>ticker</t>
   </si>
@@ -28,56 +28,50 @@
     <t>quantity</t>
   </si>
   <si>
-    <t>QAN.AX</t>
-  </si>
-  <si>
-    <t>HUB.AX</t>
-  </si>
-  <si>
-    <t>ORG.AX</t>
-  </si>
-  <si>
-    <t>GNP.AX</t>
-  </si>
-  <si>
-    <t>MTS.AX</t>
-  </si>
-  <si>
-    <t>QBE.AX</t>
-  </si>
-  <si>
-    <t>IAG.AX</t>
-  </si>
-  <si>
-    <t>PRN.AX</t>
-  </si>
-  <si>
-    <t>ABB.AX</t>
-  </si>
-  <si>
-    <t>SGLLV.AX</t>
-  </si>
-  <si>
-    <t>UNI.AX</t>
-  </si>
-  <si>
-    <t>ORI.AX</t>
-  </si>
-  <si>
-    <t>CAR.AX</t>
-  </si>
-  <si>
-    <t>TCO.AX</t>
-  </si>
-  <si>
-    <t>PPS.AX</t>
+    <t>BOQ.AX</t>
+  </si>
+  <si>
+    <t>GMG.AX</t>
+  </si>
+  <si>
+    <t>WES.AX</t>
+  </si>
+  <si>
+    <t>MQG.AX</t>
+  </si>
+  <si>
+    <t>HM1.AX</t>
+  </si>
+  <si>
+    <t>PIA.AX</t>
+  </si>
+  <si>
+    <t>IGL.AX</t>
+  </si>
+  <si>
+    <t>SUL.AX</t>
+  </si>
+  <si>
+    <t>TWR.AX</t>
+  </si>
+  <si>
+    <t>AGL.AX</t>
+  </si>
+  <si>
+    <t>SRV.AX</t>
+  </si>
+  <si>
+    <t>KOV.AX</t>
+  </si>
+  <si>
+    <t>DOW.AX</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -88,12 +82,6 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -118,10 +106,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -436,155 +423,137 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1784</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1">
+        <v>4279</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="1">
+        <v>10042</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="1">
+        <v>4069</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="1">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="1">
+        <v>8033</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="1">
+        <v>1208</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="1">
+        <v>1598</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" s="1">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="1">
-        <v>972</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="1">
-        <v>989</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="1">
-        <v>3289</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="1">
-        <v>2300</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="1">
-        <v>1823</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="1">
-        <v>2663</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="1">
-        <v>3474</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B10" s="1">
-        <v>1088</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B11" s="1">
-        <v>9949</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="B12" s="1">
-        <v>8634</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="1">
-        <v>4750</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="B14" s="1">
-        <v>2003</v>
+        <v>1524</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A15" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B15" s="1">
-        <v>7348</v>
-      </c>
+      <c r="B15" s="1"/>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B16" s="1">
-        <v>33578</v>
-      </c>
+      <c r="B16" s="1"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
       <c r="B17" s="1"/>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A18" s="1"/>
       <c r="B18" s="1"/>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="1"/>
       <c r="B19" s="1"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A20" s="1"/>
       <c r="B20" s="1"/>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" s="1"/>
       <c r="B21" s="1"/>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" s="1"/>
       <c r="B22" s="1"/>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" s="1"/>
       <c r="B23" s="1"/>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" s="1"/>
       <c r="B24" s="1"/>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
dev adding holdings analysis and fixing some issues
</commit_message>
<xml_diff>
--- a/active_portfolio.xlsx
+++ b/active_portfolio.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daivieth/Documents/_G8I/Development/IVP-Portfolio-Management-Utils/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{501FC132-4FAD-7F4E-9A85-24E6CBA36E8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EE1F9CA-B532-0A4E-97AA-FC4993E4C65D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="19760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -420,7 +420,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>5.38</v>
+        <v>4.6100000000000003</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -428,7 +428,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>5.38</v>
+        <v>4.6100000000000003</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -436,7 +436,7 @@
         <v>4</v>
       </c>
       <c r="B4">
-        <v>5.38</v>
+        <v>4.6100000000000003</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -444,7 +444,7 @@
         <v>5</v>
       </c>
       <c r="B5">
-        <v>5.38</v>
+        <v>4.6100000000000003</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -452,7 +452,7 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>5.38</v>
+        <v>4.6100000000000003</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -460,7 +460,7 @@
         <v>7</v>
       </c>
       <c r="B7">
-        <v>5.38</v>
+        <v>4.6100000000000003</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -468,7 +468,7 @@
         <v>8</v>
       </c>
       <c r="B8">
-        <v>5.38</v>
+        <v>4.6100000000000003</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -476,7 +476,7 @@
         <v>9</v>
       </c>
       <c r="B9">
-        <v>5.38</v>
+        <v>4.6100000000000003</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -484,7 +484,7 @@
         <v>10</v>
       </c>
       <c r="B10">
-        <v>5.38</v>
+        <v>4.6100000000000003</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -492,7 +492,7 @@
         <v>11</v>
       </c>
       <c r="B11">
-        <v>5.38</v>
+        <v>4.6100000000000003</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -500,7 +500,7 @@
         <v>12</v>
       </c>
       <c r="B12">
-        <v>5.4</v>
+        <v>4.6100000000000003</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
@@ -508,7 +508,7 @@
         <v>13</v>
       </c>
       <c r="B13">
-        <v>5.4</v>
+        <v>4.6399999999999997</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -516,7 +516,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <v>5.4</v>
+        <v>4.6500000000000004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>